<commit_message>
Draw both cores of the feeder CT
The RFQ lists one CT per phase, 1200/5/5A 5P20/5P20 -- one piece of iron
with two secondary cores. I read the count off the panel schedule and drew
one symbol. The cores feed different circuits, so the single line draws two,
which is what the customer's protection sheet shows and what the reference
drawings do.

ct_differential is its own stack row rather than a wider label on
ct_protection, because the two are separate devices as far as the drawing is
concerned: separate elevations, separate leads, and on a tie the second core
goes to the far bus's differential rather than its own.

'any_ct' -- the rule that sizes the dashed compartment -- now reads the CT
roles off the stack instead of the three names hardcoded in it. Adding this
row to a list nobody remembered would have put the new CT outside the box.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/excel/intake_substation_c.xlsx
+++ b/excel/intake_substation_c.xlsx
@@ -893,7 +893,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P17"/>
+  <dimension ref="A1:Q17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -966,30 +966,35 @@
       </c>
       <c r="K1" s="18" t="inlineStr">
         <is>
+          <t>ct_differential</t>
+        </is>
+      </c>
+      <c r="L1" s="18" t="inlineStr">
+        <is>
           <t>ct_metering</t>
         </is>
       </c>
-      <c r="L1" s="18" t="inlineStr">
+      <c r="M1" s="18" t="inlineStr">
         <is>
           <t>ct_ground</t>
         </is>
       </c>
-      <c r="M1" s="18" t="inlineStr">
+      <c r="N1" s="18" t="inlineStr">
         <is>
           <t>ct_class</t>
         </is>
       </c>
-      <c r="N1" s="18" t="inlineStr">
+      <c r="O1" s="18" t="inlineStr">
         <is>
           <t>pt</t>
         </is>
       </c>
-      <c r="O1" s="18" t="inlineStr">
+      <c r="P1" s="18" t="inlineStr">
         <is>
           <t>pt_primary_fuse</t>
         </is>
       </c>
-      <c r="P1" s="18" t="inlineStr">
+      <c r="Q1" s="18" t="inlineStr">
         <is>
           <t>destination</t>
         </is>
@@ -1046,12 +1051,17 @@
           <t>2500:5/5A (3)</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>2500:5/5A (3)</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
         <is>
           <t>5P20/5P20</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>TX "B" 40/66MVA 115/34.5KV</t>
         </is>
@@ -1081,12 +1091,12 @@
           <t>POTENTIAL TRANSFORMER BUS 1</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>34.5KV:120V</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>0.5A</t>
         </is>
@@ -1143,12 +1153,17 @@
           <t>600:5/5A (3)</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>600:5/5A (3)</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
         <is>
           <t>5P20/5P20</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t>TX AUX 1</t>
         </is>
@@ -1205,12 +1220,17 @@
           <t>1200:5/5A (3)</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>1200:5/5A (3)</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
         <is>
           <t>5P20/5P20</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr">
+      <c r="Q5" t="inlineStr">
         <is>
           <t>CTO. 13C</t>
         </is>
@@ -1267,12 +1287,17 @@
           <t>1200:5/5A (3)</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>1200:5/5A (3)</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
         <is>
           <t>5P20/5P20</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr">
+      <c r="Q6" t="inlineStr">
         <is>
           <t>CTO. C</t>
         </is>
@@ -1329,12 +1354,17 @@
           <t>1200:5/5A (3)</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>1200:5/5A (3)</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
         <is>
           <t>5P20/5P20</t>
         </is>
       </c>
-      <c r="P7" t="inlineStr">
+      <c r="Q7" t="inlineStr">
         <is>
           <t>CTO. 15B</t>
         </is>
@@ -1391,12 +1421,17 @@
           <t>2500:5/5A (3)</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>2500:5/5A (3)</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
         <is>
           <t>5P20/5P20</t>
         </is>
       </c>
-      <c r="P8" t="inlineStr">
+      <c r="Q8" t="inlineStr">
         <is>
           <t>BUS 2</t>
         </is>
@@ -1473,12 +1508,17 @@
           <t>1200:5/5A (3)</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>1200:5/5A (3)</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
         <is>
           <t>5P20/5P20</t>
         </is>
       </c>
-      <c r="P10" t="inlineStr">
+      <c r="Q10" t="inlineStr">
         <is>
           <t>CTO. 15A</t>
         </is>
@@ -1535,12 +1575,17 @@
           <t>1200:5/5A (3)</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr">
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>1200:5/5A (3)</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
         <is>
           <t>5P20/5P20</t>
         </is>
       </c>
-      <c r="P11" t="inlineStr">
+      <c r="Q11" t="inlineStr">
         <is>
           <t>CTO. 19C</t>
         </is>
@@ -1597,12 +1642,17 @@
           <t>1200:5/5A (3)</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr">
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>1200:5/5A (3)</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
         <is>
           <t>5P20/5P20</t>
         </is>
       </c>
-      <c r="P12" t="inlineStr">
+      <c r="Q12" t="inlineStr">
         <is>
           <t>CTO. 14C</t>
         </is>
@@ -1659,12 +1709,17 @@
           <t>600:5/5A (3)</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr">
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>600:5/5A (3)</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
         <is>
           <t>5P20/5P20</t>
         </is>
       </c>
-      <c r="P13" t="inlineStr">
+      <c r="Q13" t="inlineStr">
         <is>
           <t>TX AUX 2</t>
         </is>
@@ -1694,12 +1749,12 @@
           <t>POTENTIAL TRANSFORMER BUS 2</t>
         </is>
       </c>
-      <c r="N14" t="inlineStr">
+      <c r="O14" t="inlineStr">
         <is>
           <t>34.5KV:120V</t>
         </is>
       </c>
-      <c r="O14" t="inlineStr">
+      <c r="P14" t="inlineStr">
         <is>
           <t>0.5A</t>
         </is>
@@ -1756,12 +1811,17 @@
           <t>2500:5/5A (3)</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr">
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>2500:5/5A (3)</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
         <is>
           <t>5P20/5P20</t>
         </is>
       </c>
-      <c r="P15" t="inlineStr">
+      <c r="Q15" t="inlineStr">
         <is>
           <t>TX "A" 40/66MVA 115/34.5KV</t>
         </is>
@@ -1826,7 +1886,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:B27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1975,89 +2035,97 @@
     <row r="13">
       <c r="A13" s="24" t="inlineStr">
         <is>
-          <t>ct_metering</t>
+          <t>ct_differential</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Metering CT. Fill this ONLY if the cubicle really has a second CT set -- leaving it blank is what keeps one-CT feeders to one CT.</t>
+          <t>Ratio of the CT feeding bus differential, e.g. 1200:5A (3). A dual-core CT (1200/5/5A) is one device in the panel schedule and two symbols here, because the two cores feed different circuits. On a tie this is the far bus's differential.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="24" t="inlineStr">
         <is>
-          <t>ct_ground</t>
+          <t>ct_metering</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>Separate ground-fault CT, e.g. 50:5A. Motor feeders.</t>
+          <t>Metering CT. Fill this ONLY if the cubicle really has a second CT set -- leaving it blank is what keeps one-CT feeders to one CT.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="24" t="inlineStr">
         <is>
-          <t>ct_class</t>
+          <t>ct_ground</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Optional. Accuracy class stamped on every CT in this cubicle, e.g. 5P20. Leave blank to take the house default for each CT's job (5P20 protection, 0.3B1.8 metering, GND CT).</t>
+          <t>Separate ground-fault CT, e.g. 50:5A. Motor feeders.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="24" t="inlineStr">
         <is>
-          <t>pt</t>
+          <t>ct_class</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>Bus PT ratio, e.g. 14,400:120V. The cubicle that states this gets the PT branch, and its secondary feeds every relay in the lineup.</t>
+          <t>Optional. Accuracy class stamped on every CT in this cubicle, e.g. 5P20. Leave blank to take the house default for each CT's job (5P20 protection, 0.3B1.8 metering, GND CT).</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="24" t="inlineStr">
         <is>
-          <t>pt_primary_fuse</t>
+          <t>pt</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>PT primary fuse, e.g. CLF 0.5E. The secondary fuse belongs on the three-line diagram, not here.</t>
+          <t>Bus PT ratio, e.g. 14,400:120V. The cubicle that states this gets the PT branch, and its secondary feeds every relay in the lineup.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="24" t="inlineStr">
         <is>
+          <t>pt_primary_fuse</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>PT primary fuse, e.g. CLF 0.5E. The secondary fuse belongs on the three-line diagram, not here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="24" t="inlineStr">
+        <is>
           <t>destination</t>
         </is>
       </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="B19" s="7" t="inlineStr">
         <is>
           <t>Source or load text printed at the cubicle entry / exit. A future feeder is a normal feeder whose destination says so.</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="4" t="n"/>
-      <c r="B19" s="7" t="n"/>
-    </row>
     <row r="20">
-      <c r="A20" s="25" t="inlineStr">
+      <c r="A20" s="4" t="n"/>
+      <c r="B20" s="7" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="25" t="inlineStr">
         <is>
           <t>A device is drawn if and only if its cell has a value.</t>
         </is>
       </c>
-      <c r="B20" s="7" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="n"/>
       <c r="B21" s="7" t="n"/>
     </row>
     <row r="22">
@@ -2079,6 +2147,10 @@
     <row r="26">
       <c r="A26" s="4" t="n"/>
       <c r="B26" s="7" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="n"/>
+      <c r="B27" s="7" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>